<commit_message>
All new db files with the labelling based on the antibiotics list presentin vocab.
</commit_message>
<xml_diff>
--- a/llacie/database/use_this_data/cleaned.xlsx
+++ b/llacie/database/use_this_data/cleaned.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/llacie/database/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/llacie/database/use_this_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC28C1C-3045-1D4C-BE45-7C4A152CEB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741D32F5-55F7-9543-BCEA-73E5DDE780E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -670,9 +670,6 @@
     <t xml:space="preserve">cefamandole </t>
   </si>
   <si>
-    <t xml:space="preserve"> former Mandol</t>
-  </si>
-  <si>
     <t xml:space="preserve">cefonicid </t>
   </si>
   <si>
@@ -965,6 +962,9 @@
   </si>
   <si>
     <t>Retapamulin</t>
+  </si>
+  <si>
+    <t>Mandol</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1027,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -1045,16 +1045,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1764,7 +1754,7 @@
         <v>71</v>
       </c>
       <c r="C37" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1808,7 +1798,7 @@
         <v>78</v>
       </c>
       <c r="C41" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1819,7 +1809,7 @@
         <v>79</v>
       </c>
       <c r="C42" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1918,7 +1908,7 @@
         <v>96</v>
       </c>
       <c r="C51" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -1962,7 +1952,7 @@
         <v>103</v>
       </c>
       <c r="C55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -2072,7 +2062,7 @@
         <v>122</v>
       </c>
       <c r="C65" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -2094,7 +2084,7 @@
         <v>125</v>
       </c>
       <c r="C67" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
@@ -2105,7 +2095,7 @@
         <v>126</v>
       </c>
       <c r="C68" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2127,7 +2117,7 @@
         <v>129</v>
       </c>
       <c r="C70" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -2149,7 +2139,7 @@
         <v>132</v>
       </c>
       <c r="C72" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2160,10 +2150,10 @@
         <v>133</v>
       </c>
       <c r="C73" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -2174,7 +2164,7 @@
         <v>134</v>
       </c>
       <c r="C74" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -2559,7 +2549,7 @@
         <v>194</v>
       </c>
       <c r="C109" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -2647,7 +2637,7 @@
         <v>207</v>
       </c>
       <c r="C117" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -2658,7 +2648,7 @@
         <v>208</v>
       </c>
       <c r="C118" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -2702,7 +2692,7 @@
         <v>215</v>
       </c>
       <c r="C122" t="s">
-        <v>216</v>
+        <v>314</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -2710,10 +2700,10 @@
         <v>121</v>
       </c>
       <c r="B123" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C123" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -2721,10 +2711,10 @@
         <v>122</v>
       </c>
       <c r="B124" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C124" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -2732,10 +2722,10 @@
         <v>123</v>
       </c>
       <c r="B125" t="s">
+        <v>218</v>
+      </c>
+      <c r="C125" t="s">
         <v>219</v>
-      </c>
-      <c r="C125" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -2743,10 +2733,10 @@
         <v>124</v>
       </c>
       <c r="B126" t="s">
+        <v>220</v>
+      </c>
+      <c r="C126" t="s">
         <v>221</v>
-      </c>
-      <c r="C126" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -2754,10 +2744,10 @@
         <v>125</v>
       </c>
       <c r="B127" t="s">
+        <v>222</v>
+      </c>
+      <c r="C127" t="s">
         <v>223</v>
-      </c>
-      <c r="C127" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -2765,10 +2755,10 @@
         <v>126</v>
       </c>
       <c r="B128" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C128" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -2776,10 +2766,10 @@
         <v>127</v>
       </c>
       <c r="B129" t="s">
+        <v>225</v>
+      </c>
+      <c r="C129" t="s">
         <v>226</v>
-      </c>
-      <c r="C129" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -2787,10 +2777,10 @@
         <v>128</v>
       </c>
       <c r="B130" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C130" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -2798,10 +2788,10 @@
         <v>129</v>
       </c>
       <c r="B131" t="s">
+        <v>228</v>
+      </c>
+      <c r="C131" t="s">
         <v>229</v>
-      </c>
-      <c r="C131" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -2809,10 +2799,10 @@
         <v>130</v>
       </c>
       <c r="B132" t="s">
+        <v>230</v>
+      </c>
+      <c r="C132" t="s">
         <v>231</v>
-      </c>
-      <c r="C132" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -2820,10 +2810,10 @@
         <v>131</v>
       </c>
       <c r="B133" t="s">
+        <v>232</v>
+      </c>
+      <c r="C133" t="s">
         <v>233</v>
-      </c>
-      <c r="C133" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -2831,10 +2821,10 @@
         <v>132</v>
       </c>
       <c r="B134" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C134" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -2842,10 +2832,10 @@
         <v>133</v>
       </c>
       <c r="B135" t="s">
+        <v>235</v>
+      </c>
+      <c r="C135" t="s">
         <v>236</v>
-      </c>
-      <c r="C135" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -2853,10 +2843,10 @@
         <v>134</v>
       </c>
       <c r="B136" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C136" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -2864,10 +2854,10 @@
         <v>135</v>
       </c>
       <c r="B137" t="s">
+        <v>238</v>
+      </c>
+      <c r="C137" t="s">
         <v>239</v>
-      </c>
-      <c r="C137" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -2875,10 +2865,10 @@
         <v>136</v>
       </c>
       <c r="B138" t="s">
+        <v>240</v>
+      </c>
+      <c r="C138" t="s">
         <v>241</v>
-      </c>
-      <c r="C138" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -2886,10 +2876,10 @@
         <v>137</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -2897,10 +2887,10 @@
         <v>138</v>
       </c>
       <c r="B140" t="s">
+        <v>243</v>
+      </c>
+      <c r="C140" t="s">
         <v>244</v>
-      </c>
-      <c r="C140" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -2908,10 +2898,10 @@
         <v>139</v>
       </c>
       <c r="B141" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C141" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -2919,10 +2909,10 @@
         <v>140</v>
       </c>
       <c r="B142" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C142" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -2930,10 +2920,10 @@
         <v>141</v>
       </c>
       <c r="B143" t="s">
+        <v>247</v>
+      </c>
+      <c r="C143" t="s">
         <v>248</v>
-      </c>
-      <c r="C143" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -2941,10 +2931,10 @@
         <v>142</v>
       </c>
       <c r="B144" t="s">
+        <v>249</v>
+      </c>
+      <c r="C144" t="s">
         <v>250</v>
-      </c>
-      <c r="C144" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -2952,10 +2942,10 @@
         <v>143</v>
       </c>
       <c r="B145" t="s">
+        <v>251</v>
+      </c>
+      <c r="C145" t="s">
         <v>252</v>
-      </c>
-      <c r="C145" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -2963,7 +2953,7 @@
         <v>144</v>
       </c>
       <c r="B146" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C146" t="s">
         <v>3</v>
@@ -2974,10 +2964,10 @@
         <v>145</v>
       </c>
       <c r="B147" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C147" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -2985,10 +2975,10 @@
         <v>146</v>
       </c>
       <c r="B148" t="s">
+        <v>255</v>
+      </c>
+      <c r="C148" t="s">
         <v>256</v>
-      </c>
-      <c r="C148" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -2996,10 +2986,10 @@
         <v>147</v>
       </c>
       <c r="B149" t="s">
+        <v>257</v>
+      </c>
+      <c r="C149" t="s">
         <v>258</v>
-      </c>
-      <c r="C149" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -3007,10 +2997,10 @@
         <v>148</v>
       </c>
       <c r="B150" t="s">
+        <v>259</v>
+      </c>
+      <c r="C150" t="s">
         <v>260</v>
-      </c>
-      <c r="C150" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -3018,10 +3008,10 @@
         <v>149</v>
       </c>
       <c r="B151" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C151" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -3029,10 +3019,10 @@
         <v>150</v>
       </c>
       <c r="B152" t="s">
+        <v>262</v>
+      </c>
+      <c r="C152" t="s">
         <v>263</v>
-      </c>
-      <c r="C152" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -3040,10 +3030,10 @@
         <v>151</v>
       </c>
       <c r="B153" t="s">
+        <v>264</v>
+      </c>
+      <c r="C153" t="s">
         <v>265</v>
-      </c>
-      <c r="C153" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -3051,10 +3041,10 @@
         <v>152</v>
       </c>
       <c r="B154" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C154" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -3062,10 +3052,10 @@
         <v>153</v>
       </c>
       <c r="B155" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C155" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -3073,10 +3063,10 @@
         <v>154</v>
       </c>
       <c r="B156" t="s">
+        <v>268</v>
+      </c>
+      <c r="C156" t="s">
         <v>269</v>
-      </c>
-      <c r="C156" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -3084,10 +3074,10 @@
         <v>155</v>
       </c>
       <c r="B157" t="s">
+        <v>270</v>
+      </c>
+      <c r="C157" t="s">
         <v>271</v>
-      </c>
-      <c r="C157" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -3095,10 +3085,10 @@
         <v>156</v>
       </c>
       <c r="B158" t="s">
+        <v>272</v>
+      </c>
+      <c r="C158" t="s">
         <v>273</v>
-      </c>
-      <c r="C158" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -3106,7 +3096,7 @@
         <v>157</v>
       </c>
       <c r="B159" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C159" t="s">
         <v>3</v>
@@ -3117,10 +3107,10 @@
         <v>158</v>
       </c>
       <c r="B160" t="s">
+        <v>275</v>
+      </c>
+      <c r="C160" t="s">
         <v>276</v>
-      </c>
-      <c r="C160" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.2">
@@ -3128,7 +3118,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>3</v>
@@ -3139,10 +3129,10 @@
         <v>160</v>
       </c>
       <c r="B162" t="s">
+        <v>278</v>
+      </c>
+      <c r="C162" t="s">
         <v>279</v>
-      </c>
-      <c r="C162" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.2">
@@ -3150,10 +3140,10 @@
         <v>161</v>
       </c>
       <c r="B163" t="s">
+        <v>280</v>
+      </c>
+      <c r="C163" t="s">
         <v>281</v>
-      </c>
-      <c r="C163" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.2">
@@ -3161,10 +3151,10 @@
         <v>162</v>
       </c>
       <c r="B164" t="s">
+        <v>282</v>
+      </c>
+      <c r="C164" t="s">
         <v>283</v>
-      </c>
-      <c r="C164" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.2">
@@ -3172,10 +3162,10 @@
         <v>163</v>
       </c>
       <c r="B165" t="s">
+        <v>284</v>
+      </c>
+      <c r="C165" t="s">
         <v>285</v>
-      </c>
-      <c r="C165" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.2">
@@ -3183,10 +3173,10 @@
         <v>164</v>
       </c>
       <c r="B166" t="s">
+        <v>286</v>
+      </c>
+      <c r="C166" t="s">
         <v>287</v>
-      </c>
-      <c r="C166" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.2">
@@ -3194,10 +3184,10 @@
         <v>165</v>
       </c>
       <c r="B167" t="s">
+        <v>288</v>
+      </c>
+      <c r="C167" t="s">
         <v>289</v>
-      </c>
-      <c r="C167" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.2">
@@ -3205,10 +3195,10 @@
         <v>166</v>
       </c>
       <c r="B168" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C168" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.2">
@@ -3216,10 +3206,10 @@
         <v>167</v>
       </c>
       <c r="B169" t="s">
+        <v>291</v>
+      </c>
+      <c r="C169" t="s">
         <v>292</v>
-      </c>
-      <c r="C169" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.2">
@@ -3227,10 +3217,10 @@
         <v>168</v>
       </c>
       <c r="B170" t="s">
+        <v>293</v>
+      </c>
+      <c r="C170" t="s">
         <v>294</v>
-      </c>
-      <c r="C170" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.2">
@@ -3238,13 +3228,13 @@
         <v>169</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C171" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D171" s="2" t="s">
         <v>313</v>
-      </c>
-      <c r="D171" s="2" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.2">
@@ -3252,10 +3242,10 @@
         <v>170</v>
       </c>
       <c r="B172" t="s">
+        <v>296</v>
+      </c>
+      <c r="C172" t="s">
         <v>297</v>
-      </c>
-      <c r="C172" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.2">
@@ -3263,10 +3253,10 @@
         <v>171</v>
       </c>
       <c r="B173" t="s">
+        <v>298</v>
+      </c>
+      <c r="C173" t="s">
         <v>299</v>
-      </c>
-      <c r="C173" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.2">
@@ -3274,10 +3264,10 @@
         <v>172</v>
       </c>
       <c r="B174" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C174" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.2">
@@ -3285,10 +3275,10 @@
         <v>173</v>
       </c>
       <c r="B175" t="s">
+        <v>301</v>
+      </c>
+      <c r="C175" t="s">
         <v>302</v>
-      </c>
-      <c r="C175" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.2">
@@ -3296,19 +3286,19 @@
         <v>174</v>
       </c>
       <c r="B176" t="s">
+        <v>303</v>
+      </c>
+      <c r="C176" t="s">
         <v>304</v>
-      </c>
-      <c r="C176" t="s">
-        <v>305</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="generic name">
-      <formula>NOT(ISERROR(SEARCH("generic name",C1)))</formula>
-    </cfRule>
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="generic name">
+      <formula>NOT(ISERROR(SEARCH("generic name",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>